<commit_message>
Poblar rol_IA de casos nuevos (fallback a señal de 1a pasada web)
Los casos nuevos no estan en la recodificacion (solo baseline); se usa la
senal usa_IA de la validacion web como rol_IA con fuente 1a pasada web, para
que el analista tenga el dato en los 25 casos.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FAdgkQ1oDBgFUfZZ8wbtHw
</commit_message>
<xml_diff>
--- a/data/gates/Planilla_Casos_para_Analisis_ILIA2026.xlsx
+++ b/data/gates/Planilla_Casos_para_Analisis_ILIA2026.xlsx
@@ -1570,14 +1570,14 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>si</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>borrador (recod)</t>
+          <t>1ª pasada web</t>
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr"/>
@@ -1634,14 +1634,14 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>si</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>borrador (recod)</t>
+          <t>1ª pasada web</t>
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr"/>
@@ -1700,14 +1700,14 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>si</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>borrador (recod)</t>
+          <t>1ª pasada web</t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr"/>
@@ -1764,14 +1764,14 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>si</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>borrador (recod)</t>
+          <t>1ª pasada web</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr"/>
@@ -1828,14 +1828,14 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="G23" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>si</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>borrador (recod)</t>
+          <t>1ª pasada web</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr"/>
@@ -1892,14 +1892,14 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>si</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>borrador (recod)</t>
+          <t>1ª pasada web</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr"/>
@@ -1956,14 +1956,14 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>si</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>borrador (recod)</t>
+          <t>1ª pasada web</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr"/>
@@ -2020,14 +2020,14 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>si</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>borrador (recod)</t>
+          <t>1ª pasada web</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr"/>
@@ -2084,14 +2084,14 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>si</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>borrador (recod)</t>
+          <t>1ª pasada web</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr"/>
@@ -2148,14 +2148,14 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>si</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>borrador (recod)</t>
+          <t>1ª pasada web</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr"/>
@@ -3957,16 +3957,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G18" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H18" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G18" s="6" t="inlineStr"/>
+      <c r="H18" s="6" t="inlineStr"/>
       <c r="I18" s="6" t="inlineStr"/>
       <c r="J18" s="4" t="inlineStr">
         <is>
@@ -4018,16 +4010,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G19" s="6" t="inlineStr"/>
+      <c r="H19" s="6" t="inlineStr"/>
       <c r="I19" s="6" t="inlineStr"/>
       <c r="J19" s="4" t="inlineStr">
         <is>
@@ -4078,16 +4062,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H20" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G20" s="6" t="inlineStr"/>
+      <c r="H20" s="6" t="inlineStr"/>
       <c r="I20" s="6" t="inlineStr"/>
       <c r="J20" s="4" t="inlineStr">
         <is>
@@ -4138,16 +4114,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G21" s="6" t="inlineStr"/>
+      <c r="H21" s="6" t="inlineStr"/>
       <c r="I21" s="6" t="inlineStr"/>
       <c r="J21" s="4" t="inlineStr">
         <is>
@@ -4198,16 +4166,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H22" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G22" s="6" t="inlineStr"/>
+      <c r="H22" s="6" t="inlineStr"/>
       <c r="I22" s="6" t="inlineStr"/>
       <c r="J22" s="4" t="inlineStr">
         <is>
@@ -4258,16 +4218,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G23" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H23" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G23" s="6" t="inlineStr"/>
+      <c r="H23" s="6" t="inlineStr"/>
       <c r="I23" s="6" t="inlineStr"/>
       <c r="J23" s="4" t="inlineStr">
         <is>
@@ -4318,16 +4270,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H24" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G24" s="6" t="inlineStr"/>
+      <c r="H24" s="6" t="inlineStr"/>
       <c r="I24" s="6" t="inlineStr"/>
       <c r="J24" s="4" t="inlineStr">
         <is>
@@ -4378,16 +4322,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H25" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G25" s="6" t="inlineStr"/>
+      <c r="H25" s="6" t="inlineStr"/>
       <c r="I25" s="6" t="inlineStr"/>
       <c r="J25" s="4" t="inlineStr">
         <is>
@@ -4438,16 +4374,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H26" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G26" s="6" t="inlineStr"/>
+      <c r="H26" s="6" t="inlineStr"/>
       <c r="I26" s="6" t="inlineStr"/>
       <c r="J26" s="4" t="inlineStr">
         <is>
@@ -4498,16 +4426,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H27" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G27" s="6" t="inlineStr"/>
+      <c r="H27" s="6" t="inlineStr"/>
       <c r="I27" s="6" t="inlineStr"/>
       <c r="J27" s="4" t="inlineStr">
         <is>
@@ -4558,16 +4478,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G28" s="6" t="inlineStr"/>
+      <c r="H28" s="6" t="inlineStr"/>
       <c r="I28" s="6" t="inlineStr"/>
       <c r="J28" s="4" t="inlineStr">
         <is>
@@ -4618,16 +4530,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G29" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H29" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G29" s="6" t="inlineStr"/>
+      <c r="H29" s="6" t="inlineStr"/>
       <c r="I29" s="6" t="inlineStr"/>
       <c r="J29" s="4" t="inlineStr">
         <is>
@@ -4678,16 +4582,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G30" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H30" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G30" s="6" t="inlineStr"/>
+      <c r="H30" s="6" t="inlineStr"/>
       <c r="I30" s="6" t="inlineStr"/>
       <c r="J30" s="4" t="inlineStr">
         <is>
@@ -4738,16 +4634,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H31" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G31" s="6" t="inlineStr"/>
+      <c r="H31" s="6" t="inlineStr"/>
       <c r="I31" s="6" t="inlineStr"/>
       <c r="J31" s="4" t="inlineStr">
         <is>
@@ -4798,16 +4686,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G32" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H32" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G32" s="6" t="inlineStr"/>
+      <c r="H32" s="6" t="inlineStr"/>
       <c r="I32" s="6" t="inlineStr"/>
       <c r="J32" s="4" t="inlineStr">
         <is>
@@ -4858,16 +4738,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G33" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H33" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G33" s="6" t="inlineStr"/>
+      <c r="H33" s="6" t="inlineStr"/>
       <c r="I33" s="6" t="inlineStr"/>
       <c r="J33" s="4" t="inlineStr">
         <is>
@@ -4918,16 +4790,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G34" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H34" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G34" s="6" t="inlineStr"/>
+      <c r="H34" s="6" t="inlineStr"/>
       <c r="I34" s="6" t="inlineStr"/>
       <c r="J34" s="4" t="inlineStr">
         <is>
@@ -4978,16 +4842,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G35" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H35" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G35" s="6" t="inlineStr"/>
+      <c r="H35" s="6" t="inlineStr"/>
       <c r="I35" s="6" t="inlineStr"/>
       <c r="J35" s="4" t="inlineStr">
         <is>
@@ -5038,16 +4894,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G36" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H36" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G36" s="6" t="inlineStr"/>
+      <c r="H36" s="6" t="inlineStr"/>
       <c r="I36" s="6" t="inlineStr"/>
       <c r="J36" s="4" t="inlineStr">
         <is>
@@ -5098,16 +4946,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G37" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H37" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G37" s="6" t="inlineStr"/>
+      <c r="H37" s="6" t="inlineStr"/>
       <c r="I37" s="6" t="inlineStr"/>
       <c r="J37" s="4" t="inlineStr">
         <is>
@@ -5159,16 +4999,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G38" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H38" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G38" s="6" t="inlineStr"/>
+      <c r="H38" s="6" t="inlineStr"/>
       <c r="I38" s="6" t="inlineStr"/>
       <c r="J38" s="4" t="inlineStr">
         <is>
@@ -5219,16 +5051,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G39" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H39" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G39" s="6" t="inlineStr"/>
+      <c r="H39" s="6" t="inlineStr"/>
       <c r="I39" s="6" t="inlineStr"/>
       <c r="J39" s="4" t="inlineStr">
         <is>
@@ -5279,16 +5103,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G40" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H40" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G40" s="6" t="inlineStr"/>
+      <c r="H40" s="6" t="inlineStr"/>
       <c r="I40" s="6" t="inlineStr"/>
       <c r="J40" s="4" t="inlineStr">
         <is>
@@ -5339,16 +5155,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G41" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H41" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G41" s="6" t="inlineStr"/>
+      <c r="H41" s="6" t="inlineStr"/>
       <c r="I41" s="6" t="inlineStr"/>
       <c r="J41" s="4" t="inlineStr">
         <is>
@@ -5399,16 +5207,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G42" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H42" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G42" s="6" t="inlineStr"/>
+      <c r="H42" s="6" t="inlineStr"/>
       <c r="I42" s="6" t="inlineStr"/>
       <c r="J42" s="4" t="inlineStr">
         <is>
@@ -5459,16 +5259,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G43" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H43" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G43" s="6" t="inlineStr"/>
+      <c r="H43" s="6" t="inlineStr"/>
       <c r="I43" s="6" t="inlineStr"/>
       <c r="J43" s="4" t="inlineStr">
         <is>
@@ -5519,16 +5311,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G44" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H44" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G44" s="6" t="inlineStr"/>
+      <c r="H44" s="6" t="inlineStr"/>
       <c r="I44" s="6" t="inlineStr"/>
       <c r="J44" s="4" t="inlineStr">
         <is>
@@ -5579,16 +5363,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G45" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H45" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G45" s="6" t="inlineStr"/>
+      <c r="H45" s="6" t="inlineStr"/>
       <c r="I45" s="6" t="inlineStr"/>
       <c r="J45" s="4" t="inlineStr">
         <is>
@@ -5639,16 +5415,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G46" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H46" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G46" s="6" t="inlineStr"/>
+      <c r="H46" s="6" t="inlineStr"/>
       <c r="I46" s="6" t="inlineStr"/>
       <c r="J46" s="4" t="inlineStr">
         <is>
@@ -5699,16 +5467,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G47" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H47" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G47" s="6" t="inlineStr"/>
+      <c r="H47" s="6" t="inlineStr"/>
       <c r="I47" s="6" t="inlineStr"/>
       <c r="J47" s="4" t="inlineStr">
         <is>
@@ -5759,16 +5519,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G48" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H48" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G48" s="6" t="inlineStr"/>
+      <c r="H48" s="6" t="inlineStr"/>
       <c r="I48" s="6" t="inlineStr"/>
       <c r="J48" s="4" t="inlineStr">
         <is>
@@ -5819,16 +5571,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G49" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H49" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G49" s="6" t="inlineStr"/>
+      <c r="H49" s="6" t="inlineStr"/>
       <c r="I49" s="6" t="inlineStr"/>
       <c r="J49" s="4" t="inlineStr">
         <is>
@@ -5879,16 +5623,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G50" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H50" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G50" s="6" t="inlineStr"/>
+      <c r="H50" s="6" t="inlineStr"/>
       <c r="I50" s="6" t="inlineStr"/>
       <c r="J50" s="4" t="inlineStr">
         <is>
@@ -5939,16 +5675,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G51" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H51" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G51" s="6" t="inlineStr"/>
+      <c r="H51" s="6" t="inlineStr"/>
       <c r="I51" s="6" t="inlineStr"/>
       <c r="J51" s="4" t="inlineStr">
         <is>
@@ -5999,16 +5727,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G52" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H52" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G52" s="6" t="inlineStr"/>
+      <c r="H52" s="6" t="inlineStr"/>
       <c r="I52" s="6" t="inlineStr"/>
       <c r="J52" s="4" t="inlineStr">
         <is>
@@ -6059,16 +5779,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G53" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H53" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G53" s="6" t="inlineStr"/>
+      <c r="H53" s="6" t="inlineStr"/>
       <c r="I53" s="6" t="inlineStr"/>
       <c r="J53" s="4" t="inlineStr">
         <is>
@@ -6119,16 +5831,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G54" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H54" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G54" s="6" t="inlineStr"/>
+      <c r="H54" s="6" t="inlineStr"/>
       <c r="I54" s="6" t="inlineStr"/>
       <c r="J54" s="4" t="inlineStr">
         <is>
@@ -6179,16 +5883,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G55" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H55" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G55" s="6" t="inlineStr"/>
+      <c r="H55" s="6" t="inlineStr"/>
       <c r="I55" s="6" t="inlineStr"/>
       <c r="J55" s="4" t="inlineStr">
         <is>
@@ -6239,16 +5935,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G56" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H56" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G56" s="6" t="inlineStr"/>
+      <c r="H56" s="6" t="inlineStr"/>
       <c r="I56" s="6" t="inlineStr"/>
       <c r="J56" s="4" t="inlineStr">
         <is>
@@ -6299,16 +5987,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G57" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H57" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G57" s="6" t="inlineStr"/>
+      <c r="H57" s="6" t="inlineStr"/>
       <c r="I57" s="6" t="inlineStr"/>
       <c r="J57" s="4" t="inlineStr">
         <is>
@@ -6359,16 +6039,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G58" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H58" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G58" s="6" t="inlineStr"/>
+      <c r="H58" s="6" t="inlineStr"/>
       <c r="I58" s="6" t="inlineStr"/>
       <c r="J58" s="4" t="inlineStr">
         <is>
@@ -6419,16 +6091,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G59" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H59" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G59" s="6" t="inlineStr"/>
+      <c r="H59" s="6" t="inlineStr"/>
       <c r="I59" s="6" t="inlineStr"/>
       <c r="J59" s="4" t="inlineStr">
         <is>
@@ -6479,16 +6143,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G60" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H60" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G60" s="6" t="inlineStr"/>
+      <c r="H60" s="6" t="inlineStr"/>
       <c r="I60" s="6" t="inlineStr"/>
       <c r="J60" s="4" t="inlineStr">
         <is>
@@ -6539,16 +6195,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G61" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H61" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G61" s="6" t="inlineStr"/>
+      <c r="H61" s="6" t="inlineStr"/>
       <c r="I61" s="6" t="inlineStr"/>
       <c r="J61" s="4" t="inlineStr">
         <is>
@@ -6599,16 +6247,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G62" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H62" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G62" s="6" t="inlineStr"/>
+      <c r="H62" s="6" t="inlineStr"/>
       <c r="I62" s="6" t="inlineStr"/>
       <c r="J62" s="4" t="inlineStr">
         <is>
@@ -6659,16 +6299,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G63" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H63" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G63" s="6" t="inlineStr"/>
+      <c r="H63" s="6" t="inlineStr"/>
       <c r="I63" s="6" t="inlineStr"/>
       <c r="J63" s="4" t="inlineStr">
         <is>
@@ -6719,16 +6351,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G64" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H64" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G64" s="6" t="inlineStr"/>
+      <c r="H64" s="6" t="inlineStr"/>
       <c r="I64" s="6" t="inlineStr"/>
       <c r="J64" s="4" t="inlineStr">
         <is>
@@ -6779,16 +6403,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G65" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H65" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G65" s="6" t="inlineStr"/>
+      <c r="H65" s="6" t="inlineStr"/>
       <c r="I65" s="6" t="inlineStr"/>
       <c r="J65" s="4" t="inlineStr">
         <is>
@@ -6839,16 +6455,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G66" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H66" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G66" s="6" t="inlineStr"/>
+      <c r="H66" s="6" t="inlineStr"/>
       <c r="I66" s="6" t="inlineStr"/>
       <c r="J66" s="4" t="inlineStr">
         <is>
@@ -7117,16 +6725,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G70" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H70" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G70" s="6" t="inlineStr"/>
+      <c r="H70" s="6" t="inlineStr"/>
       <c r="I70" s="6" t="inlineStr"/>
       <c r="J70" s="4" t="inlineStr">
         <is>
@@ -7178,16 +6778,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G71" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H71" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G71" s="6" t="inlineStr"/>
+      <c r="H71" s="6" t="inlineStr"/>
       <c r="I71" s="6" t="inlineStr"/>
       <c r="J71" s="4" t="inlineStr">
         <is>
@@ -7238,16 +6830,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G72" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H72" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G72" s="6" t="inlineStr"/>
+      <c r="H72" s="6" t="inlineStr"/>
       <c r="I72" s="6" t="inlineStr"/>
       <c r="J72" s="4" t="inlineStr">
         <is>
@@ -7300,16 +6884,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G73" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H73" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G73" s="6" t="inlineStr"/>
+      <c r="H73" s="6" t="inlineStr"/>
       <c r="I73" s="6" t="inlineStr"/>
       <c r="J73" s="4" t="inlineStr">
         <is>
@@ -7360,16 +6936,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G74" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H74" s="6" t="inlineStr">
-        <is>
-          <t>borrador (recod)</t>
-        </is>
-      </c>
+      <c r="G74" s="6" t="inlineStr"/>
+      <c r="H74" s="6" t="inlineStr"/>
       <c r="I74" s="6" t="inlineStr"/>
       <c r="J74" s="4" t="inlineStr">
         <is>

</xml_diff>